<commit_message>
Liste web paneli tarafindan guncellendi
</commit_message>
<xml_diff>
--- a/liste.xlsx
+++ b/liste.xlsx
@@ -442,7 +442,11 @@
           <t>Fâtiha Suresi</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">

</xml_diff>